<commit_message>
Resultados estadísticos de red con 4Nodos. 5 instancias y 5 replicaciones
</commit_message>
<xml_diff>
--- a/Casos/problema_chatGPT/resultados_excel/instancia1.xlsx
+++ b/Casos/problema_chatGPT/resultados_excel/instancia1.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10513"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felipenoris/tmp/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Laura\OneDrive - Universidad Politécnica de Madrid\optimal_power_flow\github\Casos\problema_chatGPT\resultados_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C353BCB8-5EC8-0143-BDD3-A1B661DAACD7}" xr6:coauthVersionLast="33" xr6:coauthVersionMax="33" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFD9CAD4-9BDB-42B2-8EFC-EE100FBA5DC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="460" windowWidth="28040" windowHeight="17040" xr2:uid="{52D9C27D-0EF6-DD41-9728-0267E68F7539}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{52D9C27D-0EF6-DD41-9728-0267E68F7539}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>Concepto</t>
   </si>
@@ -58,6 +59,21 @@
   </si>
   <si>
     <t>Desviación típica del coste por instancia</t>
+  </si>
+  <si>
+    <t>Inf</t>
+  </si>
+  <si>
+    <t>NaN</t>
+  </si>
+  <si>
+    <t>MINLP</t>
+  </si>
+  <si>
+    <t>Coste de generación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En alguna de las replicaciones se encuentra el coste del MINLP, que es el óptimo. Comparar la solución de las binarias y de las potencias. </t>
   </si>
 </sst>
 </file>
@@ -113,9 +129,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -153,7 +169,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -259,7 +275,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -401,7 +417,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -409,10 +425,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF0E20E-E4D8-9B45-9C94-E89B574F109C}">
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="35.4140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -420,39 +439,39 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5">
-        <v>92.17199997901916</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
+        <v>92.171999979019162</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -460,23 +479,23 @@
         <v>52.3119547902471</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B7">
-        <v>Inf</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B8">
-        <v>Inf</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -484,12 +503,30 @@
         <v>4029.9999982099916</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>10</v>
       </c>
-      <c r="B10">
-        <v>NaN</v>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13">
+        <v>4030</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>